<commit_message>
#174 C22 update in Top Board BOM.
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Top_Board_v3.4/BOM/eSpark BOM_Top (20 Boards).xlsx
+++ b/Design-Files/LSS_Top_Board_v3.4/BOM/eSpark BOM_Top (20 Boards).xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ColeBenson-SmartMotors\Design-Files\SM_Top_Board_v3.4\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ColeBenson-SmartMotors\Design-Files\LSS_Top_Board_v3.4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -226,9 +226,6 @@
     <t>0603 .022uF 100volts X7R 10% T=0.8mm</t>
   </si>
   <si>
-    <t>220uF ±20% 63V 10mm 14.5mm 1.2A 100kHz 10000hrs 105℃ -55℃~+105℃ SMD,10x14.5mm Aluminum Electrolytic Capacitors - SMD RoHS</t>
-  </si>
-  <si>
     <t>CAP CER 0.1UF 50V X7R 0402</t>
   </si>
   <si>
@@ -367,9 +364,6 @@
     <t>Cap0805</t>
   </si>
   <si>
-    <t>VKME1451J221MV</t>
-  </si>
-  <si>
     <t>Cap1206</t>
   </si>
   <si>
@@ -550,9 +544,6 @@
     <t>TDK</t>
   </si>
   <si>
-    <t>Ymin</t>
-  </si>
-  <si>
     <t>Wurth Electronics</t>
   </si>
   <si>
@@ -854,9 +845,6 @@
   </si>
   <si>
     <t>C376821</t>
-  </si>
-  <si>
-    <t>C487391</t>
   </si>
   <si>
     <t>C307331</t>
@@ -1693,6 +1681,18 @@
   </si>
   <si>
     <t>Value</t>
+  </si>
+  <si>
+    <t>220uF 63V 225mA@100KHz ±20% SMD,D10xL10.5mm Aluminum Electrolytic Capacitors - SMD ROHS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KNSCHA </t>
+  </si>
+  <si>
+    <t>C7471900</t>
+  </si>
+  <si>
+    <t>189RV0038</t>
   </si>
 </sst>
 </file>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="50" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="51" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="52" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
@@ -3068,7 +3068,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>7</v>
@@ -3077,43 +3077,43 @@
         <v>54</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H9" s="97" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I9" s="29" t="s">
+        <v>253</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>254</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>516</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>227</v>
+      </c>
+      <c r="M9" s="31" t="s">
+        <v>255</v>
+      </c>
+      <c r="N9" s="31" t="s">
         <v>256</v>
       </c>
-      <c r="J9" s="29" t="s">
+      <c r="O9" s="31" t="s">
         <v>257</v>
       </c>
-      <c r="K9" s="30" t="s">
-        <v>520</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>230</v>
-      </c>
-      <c r="M9" s="31" t="s">
+      <c r="P9" s="31" t="s">
         <v>258</v>
       </c>
-      <c r="N9" s="31" t="s">
+      <c r="Q9" s="31" t="s">
         <v>259</v>
       </c>
-      <c r="O9" s="31" t="s">
-        <v>260</v>
-      </c>
-      <c r="P9" s="31" t="s">
-        <v>261</v>
-      </c>
-      <c r="Q9" s="31" t="s">
-        <v>262</v>
-      </c>
       <c r="R9" s="31" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -3123,7 +3123,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="54" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D10" s="37" t="s">
         <v>8</v>
@@ -3132,22 +3132,22 @@
         <v>55</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="K10" s="38" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="L10" s="37">
         <v>1</v>
@@ -3160,7 +3160,7 @@
         <v>22</v>
       </c>
       <c r="O10" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P10" s="39">
         <v>0.38819999999999999</v>
@@ -3178,31 +3178,31 @@
         <v>2</v>
       </c>
       <c r="C11" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D11" s="78" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="E11" s="79" t="s">
         <v>56</v>
       </c>
       <c r="F11" s="78" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G11" s="79" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H11" s="95" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I11" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J11" s="78" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="K11" s="79" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="L11" s="78">
         <v>12</v>
@@ -3215,7 +3215,7 @@
         <v>300</v>
       </c>
       <c r="O11" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P11" s="72">
         <v>1.4E-3</v>
@@ -3233,31 +3233,31 @@
         <v>3</v>
       </c>
       <c r="C12" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="E12" s="38" t="s">
         <v>57</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H12" s="98" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="K12" s="38" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="L12" s="71">
         <v>2</v>
@@ -3270,7 +3270,7 @@
         <v>100</v>
       </c>
       <c r="O12" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P12" s="39">
         <v>1.2999999999999999E-3</v>
@@ -3288,31 +3288,31 @@
         <v>4</v>
       </c>
       <c r="C13" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D13" s="78" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="E13" s="79" t="s">
         <v>58</v>
       </c>
       <c r="F13" s="78" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G13" s="79" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H13" s="95" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I13" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J13" s="78" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="K13" s="79" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="L13" s="82">
         <v>1</v>
@@ -3325,7 +3325,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P13" s="72">
         <v>3.5900000000000001E-2</v>
@@ -3343,31 +3343,31 @@
         <v>5</v>
       </c>
       <c r="C14" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="E14" s="38" t="s">
         <v>59</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H14" s="98" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="K14" s="38" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="L14" s="37">
         <v>6</v>
@@ -3380,7 +3380,7 @@
         <v>130</v>
       </c>
       <c r="O14" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P14" s="39">
         <v>4.0899999999999999E-2</v>
@@ -3398,31 +3398,31 @@
         <v>6</v>
       </c>
       <c r="C15" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D15" s="78" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="E15" s="79" t="s">
         <v>60</v>
       </c>
       <c r="F15" s="78" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G15" s="79" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H15" s="95" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I15" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J15" s="78" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="K15" s="79" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="L15" s="82">
         <v>1</v>
@@ -3435,7 +3435,7 @@
         <v>100</v>
       </c>
       <c r="O15" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P15" s="72">
         <v>5.8999999999999999E-3</v>
@@ -3453,31 +3453,31 @@
         <v>7</v>
       </c>
       <c r="C16" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G16" s="76" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="H16" s="99" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="K16" s="38" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="L16" s="37">
         <v>7</v>
@@ -3490,7 +3490,7 @@
         <v>150</v>
       </c>
       <c r="O16" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P16" s="39">
         <v>3.32E-2</v>
@@ -3508,7 +3508,7 @@
         <v>8</v>
       </c>
       <c r="C17" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D17" s="78" t="s">
         <v>9</v>
@@ -3517,22 +3517,22 @@
         <v>61</v>
       </c>
       <c r="F17" s="78" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G17" s="79" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H17" s="95" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I17" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J17" s="78" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="K17" s="79" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="L17" s="78">
         <v>1</v>
@@ -3545,7 +3545,7 @@
         <v>100</v>
       </c>
       <c r="O17" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P17" s="72">
         <v>3.0999999999999999E-3</v>
@@ -3563,31 +3563,31 @@
         <v>9</v>
       </c>
       <c r="C18" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D18" s="78" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E18" s="79" t="s">
         <v>62</v>
       </c>
       <c r="F18" s="78" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G18" s="84" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H18" s="95" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I18" s="78" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="J18" s="78" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="K18" s="79" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="L18" s="78">
         <v>8</v>
@@ -3600,7 +3600,7 @@
         <v>180</v>
       </c>
       <c r="O18" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P18" s="72">
         <v>3.09E-2</v>
@@ -3618,7 +3618,7 @@
         <v>10</v>
       </c>
       <c r="C19" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D19" s="37" t="s">
         <v>10</v>
@@ -3627,22 +3627,22 @@
         <v>63</v>
       </c>
       <c r="F19" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G19" s="83" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H19" s="98" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I19" s="37" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="J19" s="37" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="K19" s="38" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="L19" s="37">
         <v>1</v>
@@ -3655,7 +3655,7 @@
         <v>100</v>
       </c>
       <c r="O19" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P19" s="39">
         <v>5.3E-3</v>
@@ -3666,38 +3666,38 @@
       </c>
       <c r="R19" s="39"/>
     </row>
-    <row r="20" spans="1:18" ht="36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="24" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="105">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C20" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D20" s="78" t="s">
         <v>11</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>64</v>
+        <v>517</v>
       </c>
       <c r="F20" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G20" s="78" t="s">
-        <v>111</v>
+        <v>520</v>
       </c>
       <c r="H20" s="95" t="s">
-        <v>172</v>
+        <v>518</v>
       </c>
       <c r="I20" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J20" s="78" t="s">
-        <v>274</v>
+        <v>519</v>
       </c>
       <c r="K20" s="79" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="L20" s="78">
         <v>1</v>
@@ -3710,14 +3710,14 @@
         <v>25</v>
       </c>
       <c r="O20" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P20" s="72">
-        <v>0.22189999999999999</v>
+        <v>0.10879999999999999</v>
       </c>
       <c r="Q20" s="72">
         <f t="shared" ref="Q20" si="9">N20*P20</f>
-        <v>5.5474999999999994</v>
+        <v>2.7199999999999998</v>
       </c>
       <c r="R20" s="72"/>
     </row>
@@ -3728,31 +3728,31 @@
         <v>12</v>
       </c>
       <c r="C21" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D21" s="78" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="E21" s="79" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F21" s="78" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G21" s="79" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H21" s="95" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I21" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J21" s="78" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="K21" s="79" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="L21" s="78">
         <v>2</v>
@@ -3765,7 +3765,7 @@
         <v>100</v>
       </c>
       <c r="O21" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P21" s="72">
         <v>3.2000000000000002E-3</v>
@@ -3783,31 +3783,31 @@
         <v>13</v>
       </c>
       <c r="C22" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D22" s="37" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="E22" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G22" s="38" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H22" s="98" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I22" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J22" s="37" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="K22" s="38" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L22" s="37">
         <v>4</v>
@@ -3820,7 +3820,7 @@
         <v>100</v>
       </c>
       <c r="O22" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P22" s="39">
         <v>7.7000000000000002E-3</v>
@@ -3838,31 +3838,31 @@
         <v>14</v>
       </c>
       <c r="C23" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D23" s="37" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F23" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H23" s="98" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I23" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J23" s="37" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="K23" s="38" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="L23" s="37">
         <v>1</v>
@@ -3875,7 +3875,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P23" s="39">
         <v>3.49E-2</v>
@@ -3893,31 +3893,31 @@
         <v>15</v>
       </c>
       <c r="C24" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D24" s="78" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E24" s="79" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F24" s="78" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G24" s="79" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H24" s="95" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I24" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J24" s="78" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="K24" s="79" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="L24" s="78">
         <v>1</v>
@@ -3930,7 +3930,7 @@
         <v>40</v>
       </c>
       <c r="O24" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P24" s="72">
         <v>1.9199999999999998E-2</v>
@@ -3948,31 +3948,31 @@
         <v>16</v>
       </c>
       <c r="C25" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D25" s="37" t="s">
         <v>13</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F25" s="37" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G25" s="85">
         <v>885012205080</v>
       </c>
       <c r="H25" s="98" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="I25" s="37" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="J25" s="37" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="K25" s="38" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="L25" s="37">
         <v>1</v>
@@ -3985,7 +3985,7 @@
         <v>100</v>
       </c>
       <c r="O25" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P25" s="39">
         <v>3.0000000000000001E-3</v>
@@ -4003,31 +4003,31 @@
         <v>17</v>
       </c>
       <c r="C26" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F26" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H26" s="37" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I26" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J26" s="37" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="K26" s="37" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="L26" s="37">
         <v>1</v>
@@ -4040,7 +4040,7 @@
         <v>100</v>
       </c>
       <c r="O26" s="70" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P26" s="106">
         <v>2.5000000000000001E-3</v>
@@ -4058,31 +4058,31 @@
         <v>18</v>
       </c>
       <c r="C27" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D27" s="78" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="E27" s="78" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="F27" s="78" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="G27" s="78" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="H27" s="78" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I27" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J27" s="78" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="K27" s="78" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="L27" s="78">
         <v>1</v>
@@ -4095,7 +4095,7 @@
         <v>50</v>
       </c>
       <c r="O27" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P27" s="108">
         <v>1.0699999999999999E-2</v>
@@ -4113,31 +4113,31 @@
         <v>19</v>
       </c>
       <c r="C28" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D28" s="37" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="G28" s="37" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="H28" s="37" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I28" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J28" s="37" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="K28" s="37" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="L28" s="37">
         <v>1</v>
@@ -4150,7 +4150,7 @@
         <v>21</v>
       </c>
       <c r="O28" s="70" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P28" s="106">
         <v>0.39529999999999998</v>
@@ -4168,31 +4168,31 @@
         <v>20</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D29" s="78" t="s">
         <v>14</v>
       </c>
       <c r="E29" s="81" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="F29" s="78" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G29" s="81" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="H29" s="100" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="I29" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J29" s="78" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="K29" s="81" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="L29" s="78">
         <v>1</v>
@@ -4205,7 +4205,7 @@
         <v>100</v>
       </c>
       <c r="O29" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P29" s="72">
         <v>3.3999999999999998E-3</v>
@@ -4223,31 +4223,31 @@
         <v>21</v>
       </c>
       <c r="C30" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F30" s="37" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H30" s="98" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I30" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J30" s="37" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="K30" s="38" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="L30" s="37">
         <v>1</v>
@@ -4260,7 +4260,7 @@
         <v>30</v>
       </c>
       <c r="O30" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P30" s="39">
         <v>0.2525</v>
@@ -4278,29 +4278,29 @@
         <v>22</v>
       </c>
       <c r="C31" s="77" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D31" s="78" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="E31" s="78" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="F31" s="78" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="G31" s="78" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="H31" s="78" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="I31" s="78"/>
       <c r="J31" s="78" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="K31" s="78" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="L31" s="78">
         <v>2</v>
@@ -4313,7 +4313,7 @@
         <v>45</v>
       </c>
       <c r="O31" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P31" s="108">
         <v>0.2087</v>
@@ -4331,31 +4331,31 @@
         <v>23</v>
       </c>
       <c r="C32" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="E32" s="38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F32" s="37" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G32" s="38" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H32" s="98" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I32" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J32" s="37" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="K32" s="38" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="L32" s="37">
         <v>2</v>
@@ -4368,7 +4368,7 @@
         <v>41</v>
       </c>
       <c r="O32" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P32" s="39">
         <v>0.89410000000000001</v>
@@ -4386,31 +4386,31 @@
         <v>24</v>
       </c>
       <c r="C33" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D33" s="37" t="s">
         <v>15</v>
       </c>
       <c r="E33" s="38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F33" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G33" s="38" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H33" s="98" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I33" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J33" s="37" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="K33" s="38" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="L33" s="37">
         <v>1</v>
@@ -4423,7 +4423,7 @@
         <v>100</v>
       </c>
       <c r="O33" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P33" s="39">
         <v>3.0999999999999999E-3</v>
@@ -4441,31 +4441,31 @@
         <v>25</v>
       </c>
       <c r="C34" s="55" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D34" s="37" t="s">
         <v>16</v>
       </c>
       <c r="E34" s="38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F34" s="37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G34" s="38" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H34" s="98" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I34" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J34" s="37" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="K34" s="38" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L34" s="37">
         <v>4</v>
@@ -4478,7 +4478,7 @@
         <v>100</v>
       </c>
       <c r="O34" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P34" s="39">
         <v>5.4999999999999997E-3</v>
@@ -4496,31 +4496,31 @@
         <v>26</v>
       </c>
       <c r="C35" s="77" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D35" s="78" t="s">
         <v>17</v>
       </c>
       <c r="E35" s="79" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F35" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G35" s="79" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H35" s="95" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="I35" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J35" s="78" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="K35" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L35" s="78">
         <v>1</v>
@@ -4533,7 +4533,7 @@
         <v>30</v>
       </c>
       <c r="O35" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P35" s="72">
         <v>4.87E-2</v>
@@ -4551,31 +4551,31 @@
         <v>27</v>
       </c>
       <c r="C36" s="55" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D36" s="37" t="s">
         <v>18</v>
       </c>
       <c r="E36" s="38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F36" s="37" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G36" s="38" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="H36" s="98" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="I36" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J36" s="37" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="K36" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L36" s="37">
         <v>1</v>
@@ -4588,7 +4588,7 @@
         <v>30</v>
       </c>
       <c r="O36" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P36" s="39">
         <v>7.4300000000000005E-2</v>
@@ -4606,31 +4606,31 @@
         <v>28</v>
       </c>
       <c r="C37" s="77" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D37" s="78" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="E37" s="79" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F37" s="78" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G37" s="79" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H37" s="95" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="I37" s="78" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="J37" s="78" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="K37" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L37" s="78">
         <v>2</v>
@@ -4643,7 +4643,7 @@
         <v>60</v>
       </c>
       <c r="O37" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P37" s="72">
         <v>2.8899999999999999E-2</v>
@@ -4661,31 +4661,31 @@
         <v>29</v>
       </c>
       <c r="C38" s="88" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D38" s="89" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="E38" s="90" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="F38" s="90" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G38" s="90" t="s">
+        <v>375</v>
+      </c>
+      <c r="H38" s="101" t="s">
         <v>379</v>
       </c>
-      <c r="H38" s="101" t="s">
-        <v>383</v>
-      </c>
       <c r="I38" s="90" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J38" s="90" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="K38" s="91" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L38" s="90">
         <v>8</v>
@@ -4698,7 +4698,7 @@
         <v>165</v>
       </c>
       <c r="O38" s="92" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P38" s="91">
         <v>0.14319999999999999</v>
@@ -4716,31 +4716,31 @@
         <v>30</v>
       </c>
       <c r="C39" s="77" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D39" s="78" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="E39" s="78" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="F39" s="78" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="G39" s="78" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="H39" s="95" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I39" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J39" s="78" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="K39" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L39" s="78">
         <v>2</v>
@@ -4753,7 +4753,7 @@
         <v>45</v>
       </c>
       <c r="O39" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P39" s="39">
         <v>0.1464</v>
@@ -4779,31 +4779,31 @@
         <v>31</v>
       </c>
       <c r="C40" s="55" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D40" s="37" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="F40" s="37" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="G40" s="37" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="H40" s="37" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="I40" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J40" s="37" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="K40" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L40" s="37">
         <v>1</v>
@@ -4816,7 +4816,7 @@
         <v>30</v>
       </c>
       <c r="O40" s="70" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P40" s="106">
         <v>8.6400000000000005E-2</v>
@@ -4834,31 +4834,31 @@
         <v>32</v>
       </c>
       <c r="C41" s="77" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="D41" s="78" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="E41" s="78" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="F41" s="78" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G41" s="78" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="H41" s="78" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="I41" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J41" s="78" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="K41" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L41" s="78">
         <v>1</v>
@@ -4871,7 +4871,7 @@
         <v>25</v>
       </c>
       <c r="O41" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P41" s="108">
         <v>0.1709</v>
@@ -4889,31 +4889,31 @@
         <v>33</v>
       </c>
       <c r="C42" s="55" t="s">
+        <v>446</v>
+      </c>
+      <c r="D42" s="37" t="s">
+        <v>410</v>
+      </c>
+      <c r="E42" s="37" t="s">
+        <v>447</v>
+      </c>
+      <c r="F42" s="37" t="s">
+        <v>448</v>
+      </c>
+      <c r="G42" s="37" t="s">
         <v>450</v>
       </c>
-      <c r="D42" s="37" t="s">
-        <v>414</v>
-      </c>
-      <c r="E42" s="37" t="s">
-        <v>451</v>
-      </c>
-      <c r="F42" s="37" t="s">
-        <v>452</v>
-      </c>
-      <c r="G42" s="37" t="s">
-        <v>454</v>
-      </c>
       <c r="H42" s="37" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="I42" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J42" s="37" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="K42" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L42" s="37">
         <v>2</v>
@@ -4926,7 +4926,7 @@
         <v>45</v>
       </c>
       <c r="O42" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P42" s="106">
         <v>0.1135</v>
@@ -4944,31 +4944,31 @@
         <v>34</v>
       </c>
       <c r="C43" s="77" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="D43" s="78" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="E43" s="78" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="F43" s="78" t="s">
+        <v>448</v>
+      </c>
+      <c r="G43" s="78" t="s">
+        <v>453</v>
+      </c>
+      <c r="H43" s="37" t="s">
+        <v>480</v>
+      </c>
+      <c r="I43" s="78" t="s">
+        <v>233</v>
+      </c>
+      <c r="J43" s="78" t="s">
         <v>452</v>
       </c>
-      <c r="G43" s="78" t="s">
-        <v>457</v>
-      </c>
-      <c r="H43" s="37" t="s">
-        <v>484</v>
-      </c>
-      <c r="I43" s="78" t="s">
-        <v>236</v>
-      </c>
-      <c r="J43" s="78" t="s">
-        <v>456</v>
-      </c>
       <c r="K43" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L43" s="78">
         <v>1</v>
@@ -4981,7 +4981,7 @@
         <v>21</v>
       </c>
       <c r="O43" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P43" s="108">
         <v>5.91E-2</v>
@@ -4999,31 +4999,31 @@
         <v>35</v>
       </c>
       <c r="C44" s="55" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="D44" s="37" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="E44" s="37" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="F44" s="37" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G44" s="37" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="H44" s="37" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="I44" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J44" s="37" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="K44" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L44" s="37">
         <v>1</v>
@@ -5036,7 +5036,7 @@
         <v>25</v>
       </c>
       <c r="O44" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P44" s="106">
         <v>0.17249999999999999</v>
@@ -5054,31 +5054,31 @@
         <v>36</v>
       </c>
       <c r="C45" s="77" t="s">
+        <v>454</v>
+      </c>
+      <c r="D45" s="78" t="s">
+        <v>413</v>
+      </c>
+      <c r="E45" s="78" t="s">
         <v>458</v>
       </c>
-      <c r="D45" s="78" t="s">
-        <v>417</v>
-      </c>
-      <c r="E45" s="78" t="s">
-        <v>462</v>
-      </c>
       <c r="F45" s="78" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="G45" s="78" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="H45" s="37" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="I45" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J45" s="78" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="K45" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L45" s="78">
         <v>2</v>
@@ -5091,7 +5091,7 @@
         <v>45</v>
       </c>
       <c r="O45" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P45" s="108">
         <v>0.2072</v>
@@ -5109,31 +5109,31 @@
         <v>37</v>
       </c>
       <c r="C46" s="55" t="s">
+        <v>496</v>
+      </c>
+      <c r="D46" s="37" t="s">
+        <v>492</v>
+      </c>
+      <c r="E46" s="37" t="s">
+        <v>497</v>
+      </c>
+      <c r="F46" s="37" t="s">
+        <v>498</v>
+      </c>
+      <c r="G46" s="37" t="s">
+        <v>483</v>
+      </c>
+      <c r="H46" s="37" t="s">
+        <v>499</v>
+      </c>
+      <c r="I46" s="37" t="s">
+        <v>233</v>
+      </c>
+      <c r="J46" s="37" t="s">
         <v>500</v>
       </c>
-      <c r="D46" s="37" t="s">
-        <v>496</v>
-      </c>
-      <c r="E46" s="37" t="s">
-        <v>501</v>
-      </c>
-      <c r="F46" s="37" t="s">
-        <v>502</v>
-      </c>
-      <c r="G46" s="37" t="s">
-        <v>487</v>
-      </c>
-      <c r="H46" s="37" t="s">
-        <v>503</v>
-      </c>
-      <c r="I46" s="37" t="s">
-        <v>236</v>
-      </c>
-      <c r="J46" s="37" t="s">
-        <v>504</v>
-      </c>
       <c r="K46" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L46" s="37">
         <v>1</v>
@@ -5146,7 +5146,7 @@
         <v>50</v>
       </c>
       <c r="O46" s="70" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P46" s="106">
         <v>1.41E-2</v>
@@ -5164,31 +5164,31 @@
         <v>38</v>
       </c>
       <c r="C47" s="77" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D47" s="78" t="s">
         <v>19</v>
       </c>
       <c r="E47" s="79" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F47" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G47" s="84" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H47" s="95" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="I47" s="78" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="J47" s="78" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="K47" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L47" s="78">
         <v>1</v>
@@ -5201,7 +5201,7 @@
         <v>30</v>
       </c>
       <c r="O47" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P47" s="72">
         <v>5.6000000000000001E-2</v>
@@ -5219,31 +5219,31 @@
         <v>39</v>
       </c>
       <c r="C48" s="55" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D48" s="37" t="s">
         <v>20</v>
       </c>
       <c r="E48" s="38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F48" s="37" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="G48" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H48" s="98" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I48" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J48" s="37" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="K48" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L48" s="37">
         <v>4</v>
@@ -5256,7 +5256,7 @@
         <v>100</v>
       </c>
       <c r="O48" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P48" s="39">
         <v>2.9499999999999998E-2</v>
@@ -5274,31 +5274,31 @@
         <v>40</v>
       </c>
       <c r="C49" s="77" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="D49" s="71" t="s">
         <v>21</v>
       </c>
       <c r="E49" s="37" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="F49" s="37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G49" s="37" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="H49" s="37" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="I49" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J49" s="78" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="K49" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L49" s="78">
         <v>1</v>
@@ -5311,7 +5311,7 @@
         <v>21</v>
       </c>
       <c r="O49" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P49" s="72">
         <v>0.53559999999999997</v>
@@ -5329,31 +5329,31 @@
         <v>41</v>
       </c>
       <c r="C50" s="77" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="D50" s="82" t="s">
         <v>22</v>
       </c>
       <c r="E50" s="78" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="F50" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G50" s="78" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="H50" s="95" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="I50" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J50" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K50" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L50" s="78">
         <v>2</v>
@@ -5366,7 +5366,7 @@
         <v>42</v>
       </c>
       <c r="O50" s="57" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="P50" s="39">
         <v>2.2490000000000001</v>
@@ -5384,31 +5384,31 @@
         <v>42</v>
       </c>
       <c r="C51" s="77" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D51" s="78" t="s">
         <v>23</v>
       </c>
       <c r="E51" s="79" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F51" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G51" s="79" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H51" s="95" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="I51" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J51" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K51" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L51" s="78">
         <v>1</v>
@@ -5421,7 +5421,7 @@
         <v>21</v>
       </c>
       <c r="O51" s="80" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="P51" s="72">
         <v>1.2</v>
@@ -5439,31 +5439,31 @@
         <v>43</v>
       </c>
       <c r="C52" s="55" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D52" s="37" t="s">
         <v>24</v>
       </c>
       <c r="E52" s="38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F52" s="37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G52" s="38" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H52" s="98" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="I52" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J52" s="37" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="K52" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L52" s="37">
         <v>1</v>
@@ -5476,7 +5476,7 @@
         <v>30</v>
       </c>
       <c r="O52" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P52" s="39">
         <v>4.65E-2</v>
@@ -5494,31 +5494,31 @@
         <v>44</v>
       </c>
       <c r="C53" s="55" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="D53" s="37" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="E53" s="37" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="F53" s="37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G53" s="37">
         <v>533980367</v>
       </c>
       <c r="H53" s="98" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="I53" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J53" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K53" s="39" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L53" s="37">
         <v>1</v>
@@ -5531,7 +5531,7 @@
         <v>21</v>
       </c>
       <c r="O53" s="57" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="P53" s="39">
         <v>1.167</v>
@@ -5549,31 +5549,31 @@
         <v>45</v>
       </c>
       <c r="C54" s="55" t="s">
+        <v>392</v>
+      </c>
+      <c r="D54" s="78" t="s">
         <v>396</v>
       </c>
-      <c r="D54" s="78" t="s">
+      <c r="E54" s="78" t="s">
+        <v>398</v>
+      </c>
+      <c r="F54" s="78" t="s">
+        <v>228</v>
+      </c>
+      <c r="G54" s="78" t="s">
+        <v>397</v>
+      </c>
+      <c r="H54" s="78" t="s">
+        <v>399</v>
+      </c>
+      <c r="I54" s="37" t="s">
+        <v>233</v>
+      </c>
+      <c r="J54" s="37" t="s">
         <v>400</v>
       </c>
-      <c r="E54" s="78" t="s">
-        <v>402</v>
-      </c>
-      <c r="F54" s="78" t="s">
-        <v>231</v>
-      </c>
-      <c r="G54" s="78" t="s">
-        <v>401</v>
-      </c>
-      <c r="H54" s="78" t="s">
-        <v>403</v>
-      </c>
-      <c r="I54" s="37" t="s">
-        <v>236</v>
-      </c>
-      <c r="J54" s="37" t="s">
-        <v>404</v>
-      </c>
       <c r="K54" s="39" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L54" s="37">
         <v>1</v>
@@ -5586,7 +5586,7 @@
         <v>20</v>
       </c>
       <c r="O54" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P54" s="39">
         <v>6.8699999999999997E-2</v>
@@ -5604,31 +5604,31 @@
         <v>46</v>
       </c>
       <c r="C55" s="77" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="D55" s="82" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="E55" s="78" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="F55" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G55" s="78" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="H55" s="95" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="I55" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J55" s="78" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="K55" s="72" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L55" s="78">
         <v>1</v>
@@ -5641,7 +5641,7 @@
         <v>25</v>
       </c>
       <c r="O55" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P55" s="39">
         <v>0.2044</v>
@@ -5659,31 +5659,31 @@
         <v>47</v>
       </c>
       <c r="C56" s="77" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D56" s="78" t="s">
         <v>25</v>
       </c>
       <c r="E56" s="79" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F56" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G56" s="79" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H56" s="95" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I56" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J56" s="78" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="K56" s="79" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="L56" s="78">
         <v>1</v>
@@ -5696,7 +5696,7 @@
         <v>21</v>
       </c>
       <c r="O56" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P56" s="72">
         <v>0.45629999999999998</v>
@@ -5714,31 +5714,31 @@
         <v>48</v>
       </c>
       <c r="C57" s="55" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D57" s="37" t="s">
         <v>26</v>
       </c>
       <c r="E57" s="38" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="F57" s="37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G57" s="38" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="H57" s="98" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="I57" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J57" s="37" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="K57" s="38" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="L57" s="37">
         <v>1</v>
@@ -5751,7 +5751,7 @@
         <v>25</v>
       </c>
       <c r="O57" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P57" s="39">
         <v>0.1012</v>
@@ -5769,31 +5769,31 @@
         <v>49</v>
       </c>
       <c r="C58" s="77" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D58" s="78" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="E58" s="78" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="F58" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G58" s="78" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="H58" s="78" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="I58" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J58" s="78" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="K58" s="78" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="L58" s="78">
         <v>1</v>
@@ -5806,7 +5806,7 @@
         <v>30</v>
       </c>
       <c r="O58" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P58" s="108">
         <v>3.9199999999999999E-2</v>
@@ -5824,31 +5824,31 @@
         <v>50</v>
       </c>
       <c r="C59" s="77" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D59" s="78" t="s">
         <v>27</v>
       </c>
       <c r="E59" s="79" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F59" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G59" s="79" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H59" s="95" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I59" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J59" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K59" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L59" s="78">
         <v>1</v>
@@ -5861,7 +5861,7 @@
         <v>30</v>
       </c>
       <c r="O59" s="80" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="P59" s="72">
         <v>0.156</v>
@@ -5879,31 +5879,31 @@
         <v>51</v>
       </c>
       <c r="C60" s="55" t="s">
+        <v>352</v>
+      </c>
+      <c r="D60" s="37" t="s">
+        <v>233</v>
+      </c>
+      <c r="E60" s="38" t="s">
+        <v>354</v>
+      </c>
+      <c r="F60" s="37" t="s">
+        <v>228</v>
+      </c>
+      <c r="G60" s="38" t="s">
+        <v>355</v>
+      </c>
+      <c r="H60" s="98" t="s">
         <v>356</v>
       </c>
-      <c r="D60" s="37" t="s">
-        <v>236</v>
-      </c>
-      <c r="E60" s="38" t="s">
-        <v>358</v>
-      </c>
-      <c r="F60" s="37" t="s">
-        <v>231</v>
-      </c>
-      <c r="G60" s="38" t="s">
-        <v>359</v>
-      </c>
-      <c r="H60" s="98" t="s">
-        <v>360</v>
-      </c>
       <c r="I60" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J60" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K60" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L60" s="37">
         <v>1</v>
@@ -5916,7 +5916,7 @@
         <v>20</v>
       </c>
       <c r="O60" s="57" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="P60" s="39">
         <v>0.435</v>
@@ -5926,7 +5926,7 @@
         <v>8.6999999999999993</v>
       </c>
       <c r="R60" s="69" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.25">
@@ -5936,31 +5936,31 @@
         <v>52</v>
       </c>
       <c r="C61" s="77" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D61" s="78" t="s">
         <v>28</v>
       </c>
       <c r="E61" s="79" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F61" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G61" s="79" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H61" s="95" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="I61" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J61" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K61" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L61" s="78">
         <v>2</v>
@@ -5973,7 +5973,7 @@
         <v>42</v>
       </c>
       <c r="O61" s="80" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="P61" s="72">
         <v>1.58</v>
@@ -5991,31 +5991,31 @@
         <v>53</v>
       </c>
       <c r="C62" s="73" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D62" s="74" t="s">
         <v>29</v>
       </c>
       <c r="E62" s="75" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F62" s="74" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G62" s="74" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H62" s="102" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I62" s="74" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J62" s="74" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K62" s="75" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L62" s="74">
         <v>4</v>
@@ -6029,16 +6029,16 @@
         <v>88</v>
       </c>
       <c r="O62" s="58" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="P62" s="58" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="Q62" s="58" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="R62" s="58" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
     </row>
     <row r="63" spans="1:18" ht="36" x14ac:dyDescent="0.25">
@@ -6048,31 +6048,31 @@
         <v>54</v>
       </c>
       <c r="C63" s="55" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D63" s="37" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="E63" s="37" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="F63" s="37" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="G63" s="37" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="H63" s="98" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="I63" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J63" s="37" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="K63" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L63" s="37">
         <v>4</v>
@@ -6085,7 +6085,7 @@
         <v>85</v>
       </c>
       <c r="O63" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P63" s="39">
         <v>0.21740000000000001</v>
@@ -6103,31 +6103,31 @@
         <v>55</v>
       </c>
       <c r="C64" s="77" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="D64" s="78" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="E64" s="78" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="F64" s="78" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="G64" s="78" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="H64" s="78" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="I64" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J64" s="78" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="K64" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L64" s="78">
         <v>1</v>
@@ -6140,7 +6140,7 @@
         <v>21</v>
       </c>
       <c r="O64" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P64" s="108">
         <v>1.6523000000000001</v>
@@ -6158,31 +6158,31 @@
         <v>56</v>
       </c>
       <c r="C65" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D65" s="78" t="s">
         <v>30</v>
       </c>
       <c r="E65" s="79" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F65" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G65" s="79" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H65" s="95" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I65" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J65" s="78" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="K65" s="79" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="L65" s="78">
         <v>2</v>
@@ -6195,7 +6195,7 @@
         <v>100</v>
       </c>
       <c r="O65" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P65" s="72">
         <v>1E-3</v>
@@ -6213,31 +6213,31 @@
         <v>57</v>
       </c>
       <c r="C66" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D66" s="37" t="s">
         <v>31</v>
       </c>
       <c r="E66" s="38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F66" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G66" s="38" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H66" s="98" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I66" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J66" s="37" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="K66" s="38" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="L66" s="37">
         <v>1</v>
@@ -6250,7 +6250,7 @@
         <v>100</v>
       </c>
       <c r="O66" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P66" s="39">
         <v>1.4E-3</v>
@@ -6268,31 +6268,31 @@
         <v>58</v>
       </c>
       <c r="C67" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D67" s="78" t="s">
         <v>32</v>
       </c>
       <c r="E67" s="79" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F67" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G67" s="79" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H67" s="95" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="I67" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J67" s="78" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="K67" s="79" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="L67" s="78">
         <v>1</v>
@@ -6305,7 +6305,7 @@
         <v>100</v>
       </c>
       <c r="O67" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P67" s="72">
         <v>1.6000000000000001E-3</v>
@@ -6323,31 +6323,31 @@
         <v>59</v>
       </c>
       <c r="C68" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D68" s="37" t="s">
         <v>33</v>
       </c>
       <c r="E68" s="38" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F68" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G68" s="38" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H68" s="98" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I68" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J68" s="37" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="K68" s="38" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="L68" s="37">
         <v>2</v>
@@ -6360,7 +6360,7 @@
         <v>100</v>
       </c>
       <c r="O68" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P68" s="39">
         <v>1.4E-3</v>
@@ -6378,31 +6378,31 @@
         <v>60</v>
       </c>
       <c r="C69" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D69" s="78" t="s">
         <v>34</v>
       </c>
       <c r="E69" s="79" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F69" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G69" s="79" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H69" s="95" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I69" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J69" s="78" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="K69" s="79" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="L69" s="78">
         <v>4</v>
@@ -6415,7 +6415,7 @@
         <v>100</v>
       </c>
       <c r="O69" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P69" s="72">
         <v>1.2999999999999999E-3</v>
@@ -6433,31 +6433,31 @@
         <v>61</v>
       </c>
       <c r="C70" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D70" s="78" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="E70" s="78" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="F70" s="78" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="G70" s="78" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="H70" s="78" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I70" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J70" s="78" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="K70" s="78" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="L70" s="78">
         <v>1</v>
@@ -6470,7 +6470,7 @@
         <v>100</v>
       </c>
       <c r="O70" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P70" s="108">
         <v>8.9999999999999998E-4</v>
@@ -6488,31 +6488,31 @@
         <v>62</v>
       </c>
       <c r="C71" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D71" s="37" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="E71" s="37" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="F71" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G71" s="37" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="H71" s="37" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I71" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J71" s="37" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="K71" s="37" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="L71" s="37">
         <v>1</v>
@@ -6525,7 +6525,7 @@
         <v>40</v>
       </c>
       <c r="O71" s="70" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P71" s="106">
         <v>2.5999999999999999E-2</v>
@@ -6543,31 +6543,31 @@
         <v>63</v>
       </c>
       <c r="C72" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D72" s="37" t="s">
+        <v>362</v>
+      </c>
+      <c r="E72" s="78" t="s">
+        <v>363</v>
+      </c>
+      <c r="F72" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="G72" s="37" t="s">
+        <v>364</v>
+      </c>
+      <c r="H72" s="98" t="s">
+        <v>181</v>
+      </c>
+      <c r="I72" s="37" t="s">
+        <v>233</v>
+      </c>
+      <c r="J72" s="37" t="s">
+        <v>365</v>
+      </c>
+      <c r="K72" s="38" t="s">
         <v>366</v>
-      </c>
-      <c r="E72" s="78" t="s">
-        <v>367</v>
-      </c>
-      <c r="F72" s="37" t="s">
-        <v>125</v>
-      </c>
-      <c r="G72" s="37" t="s">
-        <v>368</v>
-      </c>
-      <c r="H72" s="98" t="s">
-        <v>184</v>
-      </c>
-      <c r="I72" s="37" t="s">
-        <v>236</v>
-      </c>
-      <c r="J72" s="37" t="s">
-        <v>369</v>
-      </c>
-      <c r="K72" s="38" t="s">
-        <v>370</v>
       </c>
       <c r="L72" s="37">
         <v>2</v>
@@ -6580,7 +6580,7 @@
         <v>45</v>
       </c>
       <c r="O72" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P72" s="39">
         <v>2.9100000000000001E-2</v>
@@ -6598,31 +6598,31 @@
         <v>64</v>
       </c>
       <c r="C73" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D73" s="37" t="s">
+        <v>321</v>
+      </c>
+      <c r="E73" s="37" t="s">
+        <v>337</v>
+      </c>
+      <c r="F73" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="G73" s="37" t="s">
+        <v>323</v>
+      </c>
+      <c r="H73" s="98" t="s">
+        <v>183</v>
+      </c>
+      <c r="I73" s="37" t="s">
+        <v>233</v>
+      </c>
+      <c r="J73" s="37" t="s">
+        <v>324</v>
+      </c>
+      <c r="K73" s="39" t="s">
         <v>325</v>
-      </c>
-      <c r="E73" s="37" t="s">
-        <v>341</v>
-      </c>
-      <c r="F73" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="G73" s="37" t="s">
-        <v>327</v>
-      </c>
-      <c r="H73" s="98" t="s">
-        <v>186</v>
-      </c>
-      <c r="I73" s="37" t="s">
-        <v>236</v>
-      </c>
-      <c r="J73" s="37" t="s">
-        <v>328</v>
-      </c>
-      <c r="K73" s="39" t="s">
-        <v>329</v>
       </c>
       <c r="L73" s="37">
         <v>8</v>
@@ -6635,7 +6635,7 @@
         <v>200</v>
       </c>
       <c r="O73" s="70" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P73" s="37">
         <v>1.1000000000000001E-3</v>
@@ -6653,31 +6653,31 @@
         <v>65</v>
       </c>
       <c r="C74" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D74" s="78" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="E74" s="78" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="F74" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G74" s="78" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="H74" s="78" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I74" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J74" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K74" s="78" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="L74" s="78">
         <v>2</v>
@@ -6690,7 +6690,7 @@
         <v>41</v>
       </c>
       <c r="O74" s="109" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="P74" s="108">
         <v>4.9800000000000001E-3</v>
@@ -6708,31 +6708,31 @@
         <v>66</v>
       </c>
       <c r="C75" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D75" s="37" t="s">
         <v>35</v>
       </c>
       <c r="E75" s="37" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="F75" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G75" s="37" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="H75" s="37" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I75" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J75" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K75" s="37" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="L75" s="37">
         <v>1</v>
@@ -6745,7 +6745,7 @@
         <v>21</v>
       </c>
       <c r="O75" s="70" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="P75" s="106">
         <v>4.1999999999999997E-3</v>
@@ -6763,31 +6763,31 @@
         <v>67</v>
       </c>
       <c r="C76" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D76" s="37" t="s">
         <v>36</v>
       </c>
       <c r="E76" s="38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F76" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G76" s="38" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H76" s="98" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="I76" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J76" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K76" s="38" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="L76" s="37">
         <v>1</v>
@@ -6800,7 +6800,7 @@
         <v>50</v>
       </c>
       <c r="O76" s="57" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="P76" s="39">
         <v>4.6699999999999997E-3</v>
@@ -6818,31 +6818,31 @@
         <v>68</v>
       </c>
       <c r="C77" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D77" s="78" t="s">
         <v>37</v>
       </c>
       <c r="E77" s="79" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F77" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G77" s="84" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H77" s="95" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I77" s="78" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="J77" s="78" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="K77" s="79" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="L77" s="78">
         <v>1</v>
@@ -6855,7 +6855,7 @@
         <v>50</v>
       </c>
       <c r="O77" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P77" s="72">
         <v>6.8999999999999999E-3</v>
@@ -6873,31 +6873,31 @@
         <v>69</v>
       </c>
       <c r="C78" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D78" s="37" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="E78" s="38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F78" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G78" s="38" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H78" s="98" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I78" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J78" s="37" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="K78" s="38" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="L78" s="37">
         <v>2</v>
@@ -6910,7 +6910,7 @@
         <v>100</v>
       </c>
       <c r="O78" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P78" s="39">
         <v>1.1000000000000001E-3</v>
@@ -6928,31 +6928,31 @@
         <v>70</v>
       </c>
       <c r="C79" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D79" s="37" t="s">
         <v>38</v>
       </c>
       <c r="E79" s="38" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F79" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G79" s="38" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H79" s="98" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I79" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J79" s="37" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="K79" s="38" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="L79" s="37">
         <v>2</v>
@@ -6965,7 +6965,7 @@
         <v>100</v>
       </c>
       <c r="O79" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P79" s="39">
         <v>1.5E-3</v>
@@ -6983,29 +6983,29 @@
         <v>71</v>
       </c>
       <c r="C80" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D80" s="82" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="E80" s="79" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F80" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G80" s="79" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H80" s="95" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I80" s="78"/>
       <c r="J80" s="78" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="K80" s="79" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="L80" s="78">
         <v>1</v>
@@ -7018,7 +7018,7 @@
         <v>100</v>
       </c>
       <c r="O80" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P80" s="72">
         <v>1.5E-3</v>
@@ -7036,31 +7036,31 @@
         <v>72</v>
       </c>
       <c r="C81" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D81" s="37" t="s">
         <v>39</v>
       </c>
       <c r="E81" s="38" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F81" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G81" s="38" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H81" s="98" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I81" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J81" s="37" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="K81" s="38" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L81" s="37">
         <v>2</v>
@@ -7073,7 +7073,7 @@
         <v>100</v>
       </c>
       <c r="O81" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P81" s="39">
         <v>1.5E-3</v>
@@ -7091,31 +7091,31 @@
         <v>73</v>
       </c>
       <c r="C82" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D82" s="78" t="s">
         <v>40</v>
       </c>
       <c r="E82" s="79" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F82" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G82" s="79" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H82" s="95" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="I82" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J82" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K82" s="79" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="L82" s="78">
         <v>1</v>
@@ -7128,7 +7128,7 @@
         <v>25</v>
       </c>
       <c r="O82" s="80" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="P82" s="72">
         <v>8.5400000000000004E-2</v>
@@ -7146,44 +7146,44 @@
         <v>74</v>
       </c>
       <c r="C83" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D83" s="37" t="s">
         <v>41</v>
       </c>
       <c r="E83" s="38" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="F83" s="71" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G83" s="38" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="H83" s="98" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="I83" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J83" s="37" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="K83" s="38" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="L83" s="37">
         <v>1</v>
       </c>
       <c r="M83" s="39">
-        <f t="shared" ref="M83:M98" si="58">L83*20</f>
+        <f t="shared" ref="M83:M94" si="58">L83*20</f>
         <v>20</v>
       </c>
       <c r="N83" s="39">
         <v>50</v>
       </c>
       <c r="O83" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P83" s="39">
         <v>3.8E-3</v>
@@ -7201,31 +7201,31 @@
         <v>75</v>
       </c>
       <c r="C84" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D84" s="78" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="E84" s="79" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F84" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G84" s="79" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H84" s="95" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I84" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J84" s="78" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="K84" s="79" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="L84" s="78">
         <v>6</v>
@@ -7238,7 +7238,7 @@
         <v>200</v>
       </c>
       <c r="O84" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P84" s="72">
         <v>1.1999999999999999E-3</v>
@@ -7256,31 +7256,31 @@
         <v>76</v>
       </c>
       <c r="C85" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D85" s="37" t="s">
         <v>42</v>
       </c>
       <c r="E85" s="38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F85" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G85" s="38" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="H85" s="98" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="I85" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J85" s="37" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="K85" s="38" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="L85" s="37">
         <v>1</v>
@@ -7293,7 +7293,7 @@
         <v>100</v>
       </c>
       <c r="O85" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P85" s="39">
         <v>1E-3</v>
@@ -7311,31 +7311,31 @@
         <v>77</v>
       </c>
       <c r="C86" s="77" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D86" s="78" t="s">
         <v>43</v>
       </c>
       <c r="E86" s="79" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F86" s="78" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G86" s="79" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="H86" s="95" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="I86" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J86" s="78" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="K86" s="79" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="L86" s="78">
         <v>1</v>
@@ -7348,7 +7348,7 @@
         <v>50</v>
       </c>
       <c r="O86" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P86" s="72">
         <v>4.3E-3</v>
@@ -7366,31 +7366,31 @@
         <v>78</v>
       </c>
       <c r="C87" s="77" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D87" s="78" t="s">
         <v>44</v>
       </c>
       <c r="E87" s="79" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F87" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G87" s="78" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H87" s="95" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="I87" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J87" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K87" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L87" s="78">
         <v>1</v>
@@ -7404,7 +7404,7 @@
         <v>22</v>
       </c>
       <c r="O87" s="80" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="P87" s="72">
         <v>1.42</v>
@@ -7421,31 +7421,31 @@
         <v>79</v>
       </c>
       <c r="C88" s="55" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D88" s="37" t="s">
         <v>45</v>
       </c>
       <c r="E88" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F88" s="37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G88" s="38">
         <v>750314597</v>
       </c>
       <c r="H88" s="98" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="I88" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J88" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K88" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L88" s="37">
         <v>1</v>
@@ -7458,7 +7458,7 @@
         <v>21</v>
       </c>
       <c r="O88" s="57" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="P88" s="39">
         <v>3.81</v>
@@ -7476,31 +7476,31 @@
         <v>80</v>
       </c>
       <c r="C89" s="77" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D89" s="78" t="s">
         <v>46</v>
       </c>
       <c r="E89" s="79" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F89" s="78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G89" s="79" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H89" s="95" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I89" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J89" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K89" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L89" s="78">
         <v>1</v>
@@ -7513,7 +7513,7 @@
         <v>21</v>
       </c>
       <c r="O89" s="80" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="P89" s="72">
         <v>2.48</v>
@@ -7531,29 +7531,29 @@
         <v>81</v>
       </c>
       <c r="C90" s="55" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D90" s="82" t="s">
         <v>47</v>
       </c>
       <c r="E90" s="78" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="F90" s="78" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="G90" s="78" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="H90" s="95" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="I90" s="37"/>
       <c r="J90" s="37" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="K90" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L90" s="37">
         <v>1</v>
@@ -7566,7 +7566,7 @@
         <v>21</v>
       </c>
       <c r="O90" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P90" s="39">
         <v>0.28160000000000002</v>
@@ -7584,31 +7584,31 @@
         <v>82</v>
       </c>
       <c r="C91" s="77" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D91" s="71" t="s">
         <v>48</v>
       </c>
       <c r="E91" s="37" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="F91" s="37" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="G91" s="37" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="H91" s="98" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="I91" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J91" s="78" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="K91" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L91" s="78">
         <v>1</v>
@@ -7621,7 +7621,7 @@
         <v>21</v>
       </c>
       <c r="O91" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P91" s="72">
         <v>0.30709999999999998</v>
@@ -7639,31 +7639,31 @@
         <v>83</v>
       </c>
       <c r="C92" s="55" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D92" s="37" t="s">
         <v>49</v>
       </c>
       <c r="E92" s="38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F92" s="37" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="G92" s="38" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H92" s="98" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I92" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J92" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K92" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L92" s="37">
         <v>1</v>
@@ -7676,7 +7676,7 @@
         <v>21</v>
       </c>
       <c r="O92" s="57" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="P92" s="39">
         <v>3.637</v>
@@ -7694,31 +7694,31 @@
         <v>84</v>
       </c>
       <c r="C93" s="77" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D93" s="78" t="s">
         <v>50</v>
       </c>
       <c r="E93" s="79" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F93" s="78" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G93" s="79" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H93" s="95" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I93" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J93" s="78" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="K93" s="79" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L93" s="78">
         <v>1</v>
@@ -7731,7 +7731,7 @@
         <v>25</v>
       </c>
       <c r="O93" s="80" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P93" s="72">
         <v>0.3463</v>
@@ -7749,31 +7749,31 @@
         <v>85</v>
       </c>
       <c r="C94" s="63" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D94" s="64" t="s">
         <v>51</v>
       </c>
       <c r="E94" s="65" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F94" s="64" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G94" s="65" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H94" s="103" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I94" s="64" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J94" s="64" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="K94" s="65" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L94" s="64">
         <v>1</v>
@@ -7786,7 +7786,7 @@
         <v>21</v>
       </c>
       <c r="O94" s="67" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P94" s="66">
         <v>7.4638</v>
@@ -7796,7 +7796,7 @@
         <v>156.7398</v>
       </c>
       <c r="R94" s="66" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
     </row>
     <row r="95" spans="1:18" x14ac:dyDescent="0.25">
@@ -7806,31 +7806,31 @@
         <v>86</v>
       </c>
       <c r="C95" s="55" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D95" s="37" t="s">
         <v>52</v>
       </c>
       <c r="E95" s="37" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="F95" s="37" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="G95" s="37" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="H95" s="37" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="I95" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J95" s="37" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="K95" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L95" s="37">
         <v>1</v>
@@ -7843,7 +7843,7 @@
         <v>21</v>
       </c>
       <c r="O95" s="70" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P95" s="106">
         <v>2.6154999999999999</v>
@@ -7861,31 +7861,31 @@
         <v>87</v>
       </c>
       <c r="C96" s="77" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D96" s="78" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="E96" s="78" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="F96" s="78" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="G96" s="78" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="H96" s="98" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I96" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J96" s="78" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="K96" s="78" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L96" s="78">
         <v>1</v>
@@ -7898,7 +7898,7 @@
         <v>21</v>
       </c>
       <c r="O96" s="109" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P96" s="108">
         <v>6.2301000000000002</v>
@@ -7916,31 +7916,31 @@
         <v>88</v>
       </c>
       <c r="C97" s="55" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D97" s="37" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="E97" s="37" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="F97" s="37" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G97" s="37" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="H97" s="98" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I97" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J97" s="37" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="K97" s="37" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L97" s="37">
         <v>1</v>
@@ -7953,7 +7953,7 @@
         <v>21</v>
       </c>
       <c r="O97" s="70" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P97" s="106">
         <v>4.7154999999999996</v>
@@ -7971,31 +7971,31 @@
         <v>89</v>
       </c>
       <c r="C98" s="55" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D98" s="37" t="s">
         <v>53</v>
       </c>
       <c r="E98" s="38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F98" s="37" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="G98" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H98" s="98" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I98" s="96" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J98" s="96" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="K98" s="38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="L98" s="37">
         <v>1</v>
@@ -8008,7 +8008,7 @@
         <v>21</v>
       </c>
       <c r="O98" s="57" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P98" s="39">
         <v>0.39140000000000003</v>
@@ -8037,12 +8037,12 @@
       <c r="M99" s="36"/>
       <c r="N99" s="36"/>
       <c r="O99" s="61" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="P99" s="59"/>
       <c r="Q99" s="59">
         <f>SUM(Q10:Q98)</f>
-        <v>1166.43948</v>
+        <v>1163.6119800000001</v>
       </c>
       <c r="R99" s="41"/>
     </row>
@@ -8064,12 +8064,12 @@
       <c r="M100" s="9"/>
       <c r="N100" s="9"/>
       <c r="O100" s="62" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="P100" s="60"/>
       <c r="Q100" s="104">
         <f>Q99/20</f>
-        <v>58.321973999999997</v>
+        <v>58.180599000000008</v>
       </c>
       <c r="R100" s="42"/>
     </row>
@@ -8106,83 +8106,83 @@
     <hyperlink ref="O17" r:id="rId7"/>
     <hyperlink ref="O18" r:id="rId8"/>
     <hyperlink ref="O19" r:id="rId9"/>
-    <hyperlink ref="O20" r:id="rId10"/>
-    <hyperlink ref="O22" r:id="rId11"/>
-    <hyperlink ref="O23" r:id="rId12"/>
-    <hyperlink ref="O24" r:id="rId13"/>
-    <hyperlink ref="O25" r:id="rId14"/>
-    <hyperlink ref="O21" r:id="rId15"/>
-    <hyperlink ref="O29" r:id="rId16"/>
-    <hyperlink ref="O30" r:id="rId17"/>
-    <hyperlink ref="O32" r:id="rId18"/>
-    <hyperlink ref="O33" r:id="rId19"/>
-    <hyperlink ref="O34" r:id="rId20"/>
-    <hyperlink ref="O35" r:id="rId21"/>
-    <hyperlink ref="O36" r:id="rId22"/>
-    <hyperlink ref="O37" r:id="rId23"/>
-    <hyperlink ref="O47" r:id="rId24"/>
-    <hyperlink ref="O48" r:id="rId25"/>
-    <hyperlink ref="O49" r:id="rId26"/>
-    <hyperlink ref="O51" r:id="rId27"/>
-    <hyperlink ref="O52" r:id="rId28"/>
-    <hyperlink ref="O56" r:id="rId29"/>
-    <hyperlink ref="O57" r:id="rId30"/>
-    <hyperlink ref="O59" r:id="rId31"/>
-    <hyperlink ref="O63" r:id="rId32"/>
-    <hyperlink ref="O65" r:id="rId33"/>
-    <hyperlink ref="O66" r:id="rId34"/>
-    <hyperlink ref="O67" r:id="rId35"/>
-    <hyperlink ref="O68" r:id="rId36"/>
-    <hyperlink ref="O69" r:id="rId37"/>
-    <hyperlink ref="O80" r:id="rId38"/>
-    <hyperlink ref="O76" r:id="rId39"/>
-    <hyperlink ref="O77" r:id="rId40"/>
-    <hyperlink ref="O78" r:id="rId41"/>
-    <hyperlink ref="O79" r:id="rId42"/>
-    <hyperlink ref="O81" r:id="rId43"/>
-    <hyperlink ref="O82" r:id="rId44"/>
-    <hyperlink ref="O83" r:id="rId45"/>
-    <hyperlink ref="O86" r:id="rId46"/>
-    <hyperlink ref="O84" r:id="rId47"/>
-    <hyperlink ref="O88" r:id="rId48"/>
-    <hyperlink ref="O89" r:id="rId49"/>
-    <hyperlink ref="O91" r:id="rId50"/>
-    <hyperlink ref="O92" r:id="rId51"/>
-    <hyperlink ref="O93" r:id="rId52"/>
-    <hyperlink ref="O94" r:id="rId53"/>
-    <hyperlink ref="O98" r:id="rId54"/>
-    <hyperlink ref="O73" r:id="rId55"/>
-    <hyperlink ref="O10" r:id="rId56"/>
-    <hyperlink ref="O87" r:id="rId57"/>
-    <hyperlink ref="O72" r:id="rId58"/>
-    <hyperlink ref="O38" r:id="rId59"/>
-    <hyperlink ref="O39" r:id="rId60"/>
-    <hyperlink ref="O50" r:id="rId61"/>
-    <hyperlink ref="O53" r:id="rId62"/>
-    <hyperlink ref="O55" r:id="rId63"/>
-    <hyperlink ref="O61" r:id="rId64"/>
-    <hyperlink ref="O54" r:id="rId65"/>
-    <hyperlink ref="O26" r:id="rId66"/>
-    <hyperlink ref="O27" r:id="rId67"/>
-    <hyperlink ref="O28" r:id="rId68"/>
-    <hyperlink ref="O31" r:id="rId69"/>
-    <hyperlink ref="O40" r:id="rId70"/>
-    <hyperlink ref="O41" r:id="rId71"/>
-    <hyperlink ref="O42" r:id="rId72"/>
-    <hyperlink ref="O43" r:id="rId73"/>
-    <hyperlink ref="O44" r:id="rId74"/>
-    <hyperlink ref="O45" r:id="rId75"/>
-    <hyperlink ref="O58" r:id="rId76"/>
-    <hyperlink ref="O70" r:id="rId77"/>
-    <hyperlink ref="O90" r:id="rId78"/>
-    <hyperlink ref="O46" r:id="rId79"/>
-    <hyperlink ref="O64" r:id="rId80"/>
-    <hyperlink ref="O71" r:id="rId81"/>
-    <hyperlink ref="O74" r:id="rId82"/>
-    <hyperlink ref="O75" r:id="rId83"/>
-    <hyperlink ref="O95" r:id="rId84"/>
-    <hyperlink ref="O96" r:id="rId85"/>
-    <hyperlink ref="O97" r:id="rId86"/>
+    <hyperlink ref="O22" r:id="rId10"/>
+    <hyperlink ref="O23" r:id="rId11"/>
+    <hyperlink ref="O24" r:id="rId12"/>
+    <hyperlink ref="O25" r:id="rId13"/>
+    <hyperlink ref="O21" r:id="rId14"/>
+    <hyperlink ref="O29" r:id="rId15"/>
+    <hyperlink ref="O30" r:id="rId16"/>
+    <hyperlink ref="O32" r:id="rId17"/>
+    <hyperlink ref="O33" r:id="rId18"/>
+    <hyperlink ref="O34" r:id="rId19"/>
+    <hyperlink ref="O35" r:id="rId20"/>
+    <hyperlink ref="O36" r:id="rId21"/>
+    <hyperlink ref="O37" r:id="rId22"/>
+    <hyperlink ref="O47" r:id="rId23"/>
+    <hyperlink ref="O48" r:id="rId24"/>
+    <hyperlink ref="O49" r:id="rId25"/>
+    <hyperlink ref="O51" r:id="rId26"/>
+    <hyperlink ref="O52" r:id="rId27"/>
+    <hyperlink ref="O56" r:id="rId28"/>
+    <hyperlink ref="O57" r:id="rId29"/>
+    <hyperlink ref="O59" r:id="rId30"/>
+    <hyperlink ref="O63" r:id="rId31"/>
+    <hyperlink ref="O65" r:id="rId32"/>
+    <hyperlink ref="O66" r:id="rId33"/>
+    <hyperlink ref="O67" r:id="rId34"/>
+    <hyperlink ref="O68" r:id="rId35"/>
+    <hyperlink ref="O69" r:id="rId36"/>
+    <hyperlink ref="O80" r:id="rId37"/>
+    <hyperlink ref="O76" r:id="rId38"/>
+    <hyperlink ref="O77" r:id="rId39"/>
+    <hyperlink ref="O78" r:id="rId40"/>
+    <hyperlink ref="O79" r:id="rId41"/>
+    <hyperlink ref="O81" r:id="rId42"/>
+    <hyperlink ref="O82" r:id="rId43"/>
+    <hyperlink ref="O83" r:id="rId44"/>
+    <hyperlink ref="O86" r:id="rId45"/>
+    <hyperlink ref="O84" r:id="rId46"/>
+    <hyperlink ref="O88" r:id="rId47"/>
+    <hyperlink ref="O89" r:id="rId48"/>
+    <hyperlink ref="O91" r:id="rId49"/>
+    <hyperlink ref="O92" r:id="rId50"/>
+    <hyperlink ref="O93" r:id="rId51"/>
+    <hyperlink ref="O94" r:id="rId52"/>
+    <hyperlink ref="O98" r:id="rId53"/>
+    <hyperlink ref="O73" r:id="rId54"/>
+    <hyperlink ref="O10" r:id="rId55"/>
+    <hyperlink ref="O87" r:id="rId56"/>
+    <hyperlink ref="O72" r:id="rId57"/>
+    <hyperlink ref="O38" r:id="rId58"/>
+    <hyperlink ref="O39" r:id="rId59"/>
+    <hyperlink ref="O50" r:id="rId60"/>
+    <hyperlink ref="O53" r:id="rId61"/>
+    <hyperlink ref="O55" r:id="rId62"/>
+    <hyperlink ref="O61" r:id="rId63"/>
+    <hyperlink ref="O54" r:id="rId64"/>
+    <hyperlink ref="O26" r:id="rId65"/>
+    <hyperlink ref="O27" r:id="rId66"/>
+    <hyperlink ref="O28" r:id="rId67"/>
+    <hyperlink ref="O31" r:id="rId68"/>
+    <hyperlink ref="O40" r:id="rId69"/>
+    <hyperlink ref="O41" r:id="rId70"/>
+    <hyperlink ref="O42" r:id="rId71"/>
+    <hyperlink ref="O43" r:id="rId72"/>
+    <hyperlink ref="O44" r:id="rId73"/>
+    <hyperlink ref="O45" r:id="rId74"/>
+    <hyperlink ref="O58" r:id="rId75"/>
+    <hyperlink ref="O70" r:id="rId76"/>
+    <hyperlink ref="O90" r:id="rId77"/>
+    <hyperlink ref="O46" r:id="rId78"/>
+    <hyperlink ref="O64" r:id="rId79"/>
+    <hyperlink ref="O71" r:id="rId80"/>
+    <hyperlink ref="O74" r:id="rId81"/>
+    <hyperlink ref="O75" r:id="rId82"/>
+    <hyperlink ref="O95" r:id="rId83"/>
+    <hyperlink ref="O96" r:id="rId84"/>
+    <hyperlink ref="O97" r:id="rId85"/>
+    <hyperlink ref="O20" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId87"/>

</xml_diff>